<commit_message>
remove petg from 3d innovators
</commit_message>
<xml_diff>
--- a/listsorter.xlsx
+++ b/listsorter.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f75adbc1b1328d64/Documents/GitHub/us-filament-cos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="24" documentId="8_{43F61E5D-CE72-4242-B668-B64B7F72F136}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6ED0672F-4196-49C1-99D0-EE66AB2F20B5}"/>
+  <xr:revisionPtr revIDLastSave="25" documentId="8_{43F61E5D-CE72-4242-B668-B64B7F72F136}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8EA5A940-2813-40F1-BC6A-F69A41EA1B53}"/>
   <bookViews>
-    <workbookView xWindow="1830" yWindow="5310" windowWidth="38700" windowHeight="15345" xr2:uid="{9B57F534-A7CF-4819-AB34-56834F09031D}"/>
+    <workbookView xWindow="2895" yWindow="5295" windowWidth="38700" windowHeight="15345" xr2:uid="{9B57F534-A7CF-4819-AB34-56834F09031D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="105">
   <si>
     <t>ZYLtech Engineering LLC</t>
   </si>
@@ -417,6 +417,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -801,7 +805,7 @@
         <v>16</v>
       </c>
       <c r="C2" t="str">
-        <f>"["&amp;A2&amp;"]"&amp;"("&amp;B2&amp;")"</f>
+        <f t="shared" ref="C2:C27" si="0">"["&amp;A2&amp;"]"&amp;"("&amp;B2&amp;")"</f>
         <v>[3D INNOVATORS LLC](https://3dinnovatorsofficial.com/shop)</v>
       </c>
       <c r="D2" t="s">
@@ -810,12 +814,9 @@
       <c r="G2" t="s">
         <v>82</v>
       </c>
-      <c r="H2" t="s">
-        <v>82</v>
-      </c>
       <c r="R2" t="str">
         <f>"| "&amp;$C2&amp;" | "&amp;$D2&amp;" | "&amp;$E2&amp;" | "&amp;$F2&amp;" | "&amp;$G2&amp;" | "&amp;$H2&amp;" | "&amp;$I2&amp;" | "&amp;$J2&amp;" | "&amp;$K2&amp;" | "&amp;$L2&amp;" | "&amp;$M2&amp;" | "&amp;$N2&amp;" | "&amp;$O2&amp;" | "&amp;$P2&amp;" |"</f>
-        <v>| [3D INNOVATORS LLC](https://3dinnovatorsofficial.com/shop) | Celina, Ohio |  |  | X | X |  |  |  |  |  |  |  |  |</v>
+        <v>| [3D INNOVATORS LLC](https://3dinnovatorsofficial.com/shop) | Celina, Ohio |  |  | X |  |  |  |  |  |  |  |  |  |</v>
       </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.25">
@@ -826,7 +827,7 @@
         <v>13</v>
       </c>
       <c r="C3" t="str">
-        <f>"["&amp;A3&amp;"]"&amp;"("&amp;B3&amp;")"</f>
+        <f t="shared" si="0"/>
         <v>[3D-Fuel](https://www.3dfuel.com)</v>
       </c>
       <c r="D3" t="s">
@@ -842,7 +843,7 @@
         <v>82</v>
       </c>
       <c r="R3" t="str">
-        <f t="shared" ref="R3:R27" si="0">"| "&amp;$C3&amp;" | "&amp;$D3&amp;" | "&amp;$E3&amp;" | "&amp;$F3&amp;" | "&amp;$G3&amp;" | "&amp;$H3&amp;" | "&amp;$I3&amp;" | "&amp;$J3&amp;" | "&amp;$K3&amp;" | "&amp;$L3&amp;" | "&amp;$M3&amp;" | "&amp;$N3&amp;" | "&amp;$O3&amp;" | "&amp;$P3&amp;" |"</f>
+        <f t="shared" ref="R3:R27" si="1">"| "&amp;$C3&amp;" | "&amp;$D3&amp;" | "&amp;$E3&amp;" | "&amp;$F3&amp;" | "&amp;$G3&amp;" | "&amp;$H3&amp;" | "&amp;$I3&amp;" | "&amp;$J3&amp;" | "&amp;$K3&amp;" | "&amp;$L3&amp;" | "&amp;$M3&amp;" | "&amp;$N3&amp;" | "&amp;$O3&amp;" | "&amp;$P3&amp;" |"</f>
         <v>| [3D-Fuel](https://www.3dfuel.com) | Fargo, North Dakota |  |  | X | X |  | X |  |  |  |  |  |  |</v>
       </c>
     </row>
@@ -854,7 +855,7 @@
         <v>10</v>
       </c>
       <c r="C4" t="str">
-        <f>"["&amp;A4&amp;"]"&amp;"("&amp;B4&amp;")"</f>
+        <f t="shared" si="0"/>
         <v>[3DXTech](https://www.3dxtech.com)</v>
       </c>
       <c r="D4" t="s">
@@ -885,7 +886,7 @@
         <v>84</v>
       </c>
       <c r="R4" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>| [3DXTech](https://www.3dxtech.com) | Grand Rapids, Michigan |  |  | X | X | X | X | X | X |  | X |  | Peek, PEI, Ultem |</v>
       </c>
     </row>
@@ -897,7 +898,7 @@
         <v>43</v>
       </c>
       <c r="C5" t="str">
-        <f>"["&amp;A5&amp;"]"&amp;"("&amp;B5&amp;")"</f>
+        <f t="shared" si="0"/>
         <v>[Ambrosia (West 3D)](https://ambrosiafilament.com/)</v>
       </c>
       <c r="D5" t="s">
@@ -922,7 +923,7 @@
         <v>85</v>
       </c>
       <c r="R5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>| [Ambrosia (West 3D)](https://ambrosiafilament.com/) | Beaverton, Oregon | Non-US, PHA is US made |  | X | X | X | X |  |  |  |  |  | PHA |</v>
       </c>
     </row>
@@ -934,7 +935,7 @@
         <v>3</v>
       </c>
       <c r="C6" t="str">
-        <f>"["&amp;A6&amp;"]"&amp;"("&amp;B6&amp;")"</f>
+        <f t="shared" si="0"/>
         <v>[American Filament](https://americanfilament.us)</v>
       </c>
       <c r="D6" t="s">
@@ -953,7 +954,7 @@
         <v>82</v>
       </c>
       <c r="R6" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>| [American Filament](https://americanfilament.us) | Huntsville, Alabama |  |  | X | X |  | X |  |  | X |  |  |  |</v>
       </c>
     </row>
@@ -965,7 +966,7 @@
         <v>6</v>
       </c>
       <c r="C7" t="str">
-        <f>"["&amp;A7&amp;"]"&amp;"("&amp;B7&amp;")"</f>
+        <f t="shared" si="0"/>
         <v>[Atomic Filament](https://atomicfilament.com)</v>
       </c>
       <c r="D7" t="s">
@@ -990,7 +991,7 @@
         <v>82</v>
       </c>
       <c r="R7" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>| [Atomic Filament](https://atomicfilament.com) | Kendallville, Indiana |  |  | X | X | X | X | X |  |  | X |  |  |</v>
       </c>
     </row>
@@ -1002,7 +1003,7 @@
         <v>11</v>
       </c>
       <c r="C8" t="str">
-        <f>"["&amp;A8&amp;"]"&amp;"("&amp;B8&amp;")"</f>
+        <f t="shared" si="0"/>
         <v>[Coex3D](https://coex3d.com)</v>
       </c>
       <c r="D8" t="s">
@@ -1027,7 +1028,7 @@
         <v>82</v>
       </c>
       <c r="R8" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>| [Coex3D](https://coex3d.com) | Appleton, Wisconsin |  |  | X | X | X | X |  |  | X | X |  |  |</v>
       </c>
     </row>
@@ -1039,7 +1040,7 @@
         <v>103</v>
       </c>
       <c r="C9" t="str">
-        <f>"["&amp;A9&amp;"]"&amp;"("&amp;B9&amp;")"</f>
+        <f t="shared" si="0"/>
         <v>[Dancyn 3D](https://www.dancyn3dprints.com/)</v>
       </c>
       <c r="D9" t="s">
@@ -1052,7 +1053,7 @@
         <v>82</v>
       </c>
       <c r="R9" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>| [Dancyn 3D](https://www.dancyn3dprints.com/) | Whippany, NJ |  |  | X | X |  |  |  |  |  |  |  |  |</v>
       </c>
     </row>
@@ -1064,7 +1065,7 @@
         <v>53</v>
       </c>
       <c r="C10" t="str">
-        <f>"["&amp;A10&amp;"]"&amp;"("&amp;B10&amp;")"</f>
+        <f t="shared" si="0"/>
         <v>[FilaCube](https://www.filacube.com/)</v>
       </c>
       <c r="D10" t="s">
@@ -1083,7 +1084,7 @@
         <v>82</v>
       </c>
       <c r="R10" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>| [FilaCube](https://www.filacube.com/) | Houston/Katy, Texas |  |  | X | X |  | X |  |  | X |  |  |  |</v>
       </c>
     </row>
@@ -1095,7 +1096,7 @@
         <v>50</v>
       </c>
       <c r="C11" t="str">
-        <f>"["&amp;A11&amp;"]"&amp;"("&amp;B11&amp;")"</f>
+        <f t="shared" si="0"/>
         <v>[Filamatrix](https://filamatrix.com/)</v>
       </c>
       <c r="D11" t="s">
@@ -1123,7 +1124,7 @@
         <v>87</v>
       </c>
       <c r="R11" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>| [Filamatrix](https://filamatrix.com/) | Chester, Virgina |  |  | X | X | X | X |  | X |  | X |  | Kevlar Composite |</v>
       </c>
     </row>
@@ -1135,7 +1136,7 @@
         <v>4</v>
       </c>
       <c r="C12" t="str">
-        <f>"["&amp;A12&amp;"]"&amp;"("&amp;B12&amp;")"</f>
+        <f t="shared" si="0"/>
         <v>[Fusion Filaments](https://www.fusionfilaments.com)</v>
       </c>
       <c r="D12" t="s">
@@ -1157,7 +1158,7 @@
         <v>82</v>
       </c>
       <c r="R12" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>| [Fusion Filaments](https://www.fusionfilaments.com) | Maryland Heights, Missouri |  |  | X | X | X | X |  |  |  |  | X |  |</v>
       </c>
     </row>
@@ -1169,7 +1170,7 @@
         <v>15</v>
       </c>
       <c r="C13" t="str">
-        <f>"["&amp;A13&amp;"]"&amp;"("&amp;B13&amp;")"</f>
+        <f t="shared" si="0"/>
         <v>[GreenGate3D](https://greengate3d.com)</v>
       </c>
       <c r="D13" t="s">
@@ -1179,7 +1180,7 @@
         <v>82</v>
       </c>
       <c r="R13" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>| [GreenGate3D](https://greengate3d.com) | Bohemia/Long Island, New York |  |  |  | X |  |  |  |  |  |  |  |  |</v>
       </c>
     </row>
@@ -1191,7 +1192,7 @@
         <v>12</v>
       </c>
       <c r="C14" t="str">
-        <f>"["&amp;A14&amp;"]"&amp;"("&amp;B14&amp;")"</f>
+        <f t="shared" si="0"/>
         <v>[IC3D](https://www.ic3dprinters.com)</v>
       </c>
       <c r="D14" t="s">
@@ -1213,7 +1214,7 @@
         <v>82</v>
       </c>
       <c r="R14" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>| [IC3D](https://www.ic3dprinters.com) | Columbus, Ohio |  |  | X | X |  | X |  |  | X | X |  |  |</v>
       </c>
     </row>
@@ -1225,7 +1226,7 @@
         <v>94</v>
       </c>
       <c r="C15" t="str">
-        <f>"["&amp;A15&amp;"]"&amp;"("&amp;B15&amp;")"</f>
+        <f t="shared" si="0"/>
         <v>[Lumas Polymers](https://lumaspolymers.com/)</v>
       </c>
       <c r="D15" t="s">
@@ -1259,7 +1260,7 @@
         <v>91</v>
       </c>
       <c r="R15" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>| [Lumas Polymers](https://lumaspolymers.com/) | Sioux Fall, South Dakota | Chaska, Minnesota |  | X | X |  | X | X | X | X | X |  | TPE |</v>
       </c>
     </row>
@@ -1271,7 +1272,7 @@
         <v>55</v>
       </c>
       <c r="C16" t="str">
-        <f>"["&amp;A16&amp;"]"&amp;"("&amp;B16&amp;")"</f>
+        <f t="shared" si="0"/>
         <v>[MatterHackers ProSeries](https://www.matterhackers.com/store/c/pro-series-filament)</v>
       </c>
       <c r="D16" t="s">
@@ -1293,7 +1294,7 @@
         <v>82</v>
       </c>
       <c r="R16" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>| [MatterHackers ProSeries](https://www.matterhackers.com/store/c/pro-series-filament) | Lake Forest, California |  |  | X | X |  | X |  |  | X | X |  |  |</v>
       </c>
     </row>
@@ -1305,7 +1306,7 @@
         <v>14</v>
       </c>
       <c r="C17" t="str">
-        <f>"["&amp;A17&amp;"]"&amp;"("&amp;B17&amp;")"</f>
+        <f t="shared" si="0"/>
         <v>[Numakers](https://numakers.com)</v>
       </c>
       <c r="D17" t="s">
@@ -1330,7 +1331,7 @@
         <v>82</v>
       </c>
       <c r="R17" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>| [Numakers](https://numakers.com) | Richmond, Virgina | India |  | X | X | X | X |  |  | X |  |  |  |</v>
       </c>
     </row>
@@ -1342,7 +1343,7 @@
         <v>90</v>
       </c>
       <c r="C18" t="str">
-        <f>"["&amp;A18&amp;"]"&amp;"("&amp;B18&amp;")"</f>
+        <f t="shared" si="0"/>
         <v>[Paramount3D](https://www.paramount-3d.com/)</v>
       </c>
       <c r="D18" t="s">
@@ -1367,7 +1368,7 @@
         <v>92</v>
       </c>
       <c r="R18" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>| [Paramount3D](https://www.paramount-3d.com/) | Bensenville/Wood Dale, Illinois |  |  | X | X | X | X |  |  | X |  |  | FlexPLA, PVA |</v>
       </c>
     </row>
@@ -1379,7 +1380,7 @@
         <v>8</v>
       </c>
       <c r="C19" t="str">
-        <f>"["&amp;A19&amp;"]"&amp;"("&amp;B19&amp;")"</f>
+        <f t="shared" si="0"/>
         <v>[Polar Filament](https://polarfilament.com)</v>
       </c>
       <c r="D19" t="s">
@@ -1392,7 +1393,7 @@
         <v>82</v>
       </c>
       <c r="R19" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>| [Polar Filament](https://polarfilament.com) | Brighton, Michigan |  |  | X | X |  |  |  |  |  |  |  |  |</v>
       </c>
     </row>
@@ -1404,7 +1405,7 @@
         <v>5</v>
       </c>
       <c r="C20" t="str">
-        <f>"["&amp;A20&amp;"]"&amp;"("&amp;B20&amp;")"</f>
+        <f t="shared" si="0"/>
         <v>[Printed Solid](https://www.printedsolid.com)</v>
       </c>
       <c r="D20" t="s">
@@ -1423,7 +1424,7 @@
         <v>82</v>
       </c>
       <c r="R20" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>| [Printed Solid](https://www.printedsolid.com) | Newark, Delaware |  |  | X | X | X | X |  |  |  |  |  |  |</v>
       </c>
     </row>
@@ -1435,7 +1436,7 @@
         <v>48</v>
       </c>
       <c r="C21" t="str">
-        <f>"["&amp;A21&amp;"]"&amp;"("&amp;B21&amp;")"</f>
+        <f t="shared" si="0"/>
         <v>[Protopasta](https://proto-pasta.com/)</v>
       </c>
       <c r="D21" t="s">
@@ -1451,7 +1452,7 @@
         <v>82</v>
       </c>
       <c r="R21" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>| [Protopasta](https://proto-pasta.com/) | Vancouver, Washington |  |  | X | X |  |  | X |  |  |  |  |  |</v>
       </c>
     </row>
@@ -1463,7 +1464,7 @@
         <v>7</v>
       </c>
       <c r="C22" t="str">
-        <f>"["&amp;A22&amp;"]"&amp;"("&amp;B22&amp;")"</f>
+        <f t="shared" si="0"/>
         <v>[Push Plastic](https://www.pushplastic.com)</v>
       </c>
       <c r="D22" t="s">
@@ -1491,7 +1492,7 @@
         <v>82</v>
       </c>
       <c r="R22" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>| [Push Plastic](https://www.pushplastic.com) | Springdale, Arkansas |  |  | X | X |  | X | X | X | X | X |  |  |</v>
       </c>
     </row>
@@ -1503,7 +1504,7 @@
         <v>40</v>
       </c>
       <c r="C23" t="str">
-        <f>"["&amp;A23&amp;"]"&amp;"("&amp;B23&amp;")"</f>
+        <f t="shared" si="0"/>
         <v>[Tangled](https://www.tangledfilament.com/)</v>
       </c>
       <c r="D23" t="s">
@@ -1516,7 +1517,7 @@
         <v>82</v>
       </c>
       <c r="R23" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>| [Tangled](https://www.tangledfilament.com/) | Nampa/Boise, Idaho |  |  | X |  |  |  |  |  |  |  | X |  |</v>
       </c>
     </row>
@@ -1528,7 +1529,7 @@
         <v>45</v>
       </c>
       <c r="C24" t="str">
-        <f>"["&amp;A24&amp;"]"&amp;"("&amp;B24&amp;")"</f>
+        <f t="shared" si="0"/>
         <v>[Toner Plastics (Village Plastics)](https://www.villageplastics.com/)</v>
       </c>
       <c r="D24" t="s">
@@ -1559,7 +1560,7 @@
         <v>86</v>
       </c>
       <c r="R24" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>| [Toner Plastics (Village Plastics)](https://www.villageplastics.com/) | East Longmeadow, Massachusetts | Barberton, Ohio |  | X | X | X | X |  | X | X |  |  | HIPS |</v>
       </c>
     </row>
@@ -1571,7 +1572,7 @@
         <v>98</v>
       </c>
       <c r="C25" t="str">
-        <f>"["&amp;A25&amp;"]"&amp;"("&amp;B25&amp;")"</f>
+        <f t="shared" si="0"/>
         <v>[Two Step Process (Luke's Laboratory)](https://www.lukeslabonline.com/)</v>
       </c>
       <c r="D25" t="s">
@@ -1593,7 +1594,7 @@
         <v>100</v>
       </c>
       <c r="R25" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>| [Two Step Process (Luke's Laboratory)](https://www.lukeslabonline.com/) | Wrightstown, WI | China |  |  |  | X | X | X |  |  |  |  | PPC-CF, PET-CF, ABS-FR |</v>
       </c>
     </row>
@@ -1605,7 +1606,7 @@
         <v>42</v>
       </c>
       <c r="C26" t="str">
-        <f>"["&amp;A26&amp;"]"&amp;"("&amp;B26&amp;")"</f>
+        <f t="shared" si="0"/>
         <v>[Voxel](https://voxelpla.com/)</v>
       </c>
       <c r="D26" t="s">
@@ -1624,7 +1625,7 @@
         <v>82</v>
       </c>
       <c r="R26" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>| [Voxel](https://voxelpla.com/) | Garden Grove, California |  |  | X | X |  | X |  |  | X |  |  |  |</v>
       </c>
     </row>
@@ -1636,7 +1637,7 @@
         <v>9</v>
       </c>
       <c r="C27" t="str">
-        <f>"["&amp;A27&amp;"]"&amp;"("&amp;B27&amp;")"</f>
+        <f t="shared" si="0"/>
         <v>[ZYLtech Engineering LLC](https://www.zyltech.com)</v>
       </c>
       <c r="D27" t="s">
@@ -1658,7 +1659,7 @@
         <v>82</v>
       </c>
       <c r="R27" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>| [ZYLtech Engineering LLC](https://www.zyltech.com) | Houston/Spring, Texas |  |  | X | X |  | X | X |  | X |  |  |  |</v>
       </c>
     </row>

</xml_diff>